<commit_message>
Shorten register sheet name for Excel compatibility
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0162N6SK8wgniuFy66fghVap
</commit_message>
<xml_diff>
--- a/Vagamon_Round5_New_Contacts.xlsx
+++ b/Vagamon_Round5_New_Contacts.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tour Operators" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vagamon Hotels &amp; Accommodations" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Vagamon Tour Packages" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Email Verification &amp; Source Register" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification and Sources" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded Previous Contacts" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unverified Leads" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="7" state="visible" r:id="rId7"/>
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tour Operators'!$A$1:$K$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Vagamon Hotels &amp; Accommodations'!$A$1:$K$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Daily Vagamon Tour Packages'!$A$1:$L$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Email Verification &amp; Source Register'!$A$1:$G$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Verification and Sources'!$A$1:$G$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Excluded Previous Contacts'!$A$1:$C$172</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Unverified Leads'!$A$1:$H$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Summary'!$A$1:$B$9</definedName>

</xml_diff>